<commit_message>
improve system test reliability
</commit_message>
<xml_diff>
--- a/docs/test/selenium_error.xlsx
+++ b/docs/test/selenium_error.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-07-25 11:28:47</t>
+          <t>2026-07-26 00:17:57</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="H3" s="4" t="n">
-        <v>147</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" ht="25" customHeight="1">
@@ -22202,7 +22202,7 @@
       </c>
       <c r="E546" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F546" s="7" t="inlineStr">
@@ -22217,7 +22217,7 @@
       </c>
       <c r="H546" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22242,7 +22242,7 @@
       </c>
       <c r="E547" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F547" s="7" t="inlineStr">
@@ -22257,7 +22257,7 @@
       </c>
       <c r="H547" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22282,7 +22282,7 @@
       </c>
       <c r="E548" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F548" s="7" t="inlineStr">
@@ -22297,7 +22297,7 @@
       </c>
       <c r="H548" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22322,7 +22322,7 @@
       </c>
       <c r="E549" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F549" s="7" t="inlineStr">
@@ -22337,7 +22337,7 @@
       </c>
       <c r="H549" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22362,7 +22362,7 @@
       </c>
       <c r="E550" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F550" s="7" t="inlineStr">
@@ -22377,7 +22377,7 @@
       </c>
       <c r="H550" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22402,7 +22402,7 @@
       </c>
       <c r="E551" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F551" s="7" t="inlineStr">
@@ -22417,7 +22417,7 @@
       </c>
       <c r="H551" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22442,7 +22442,7 @@
       </c>
       <c r="E552" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F552" s="7" t="inlineStr">
@@ -22457,7 +22457,7 @@
       </c>
       <c r="H552" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22482,7 +22482,7 @@
       </c>
       <c r="E553" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F553" s="7" t="inlineStr">
@@ -22497,7 +22497,7 @@
       </c>
       <c r="H553" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22522,7 +22522,7 @@
       </c>
       <c r="E554" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F554" s="7" t="inlineStr">
@@ -22537,7 +22537,7 @@
       </c>
       <c r="H554" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22562,7 +22562,7 @@
       </c>
       <c r="E555" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F555" s="7" t="inlineStr">
@@ -22577,7 +22577,7 @@
       </c>
       <c r="H555" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22602,7 +22602,7 @@
       </c>
       <c r="E556" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F556" s="7" t="inlineStr">
@@ -22617,7 +22617,7 @@
       </c>
       <c r="H556" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22642,7 +22642,7 @@
       </c>
       <c r="E557" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F557" s="7" t="inlineStr">
@@ -22657,7 +22657,7 @@
       </c>
       <c r="H557" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22682,7 +22682,7 @@
       </c>
       <c r="E558" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F558" s="7" t="inlineStr">
@@ -22697,7 +22697,7 @@
       </c>
       <c r="H558" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22722,7 +22722,7 @@
       </c>
       <c r="E559" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F559" s="7" t="inlineStr">
@@ -22737,7 +22737,7 @@
       </c>
       <c r="H559" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22762,7 +22762,7 @@
       </c>
       <c r="E560" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F560" s="7" t="inlineStr">
@@ -22777,7 +22777,7 @@
       </c>
       <c r="H560" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22802,7 +22802,7 @@
       </c>
       <c r="E561" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F561" s="7" t="inlineStr">
@@ -22817,7 +22817,7 @@
       </c>
       <c r="H561" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22842,7 +22842,7 @@
       </c>
       <c r="E562" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F562" s="7" t="inlineStr">
@@ -22857,7 +22857,7 @@
       </c>
       <c r="H562" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22882,7 +22882,7 @@
       </c>
       <c r="E563" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F563" s="7" t="inlineStr">
@@ -22897,7 +22897,7 @@
       </c>
       <c r="H563" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22922,7 +22922,7 @@
       </c>
       <c r="E564" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F564" s="7" t="inlineStr">
@@ -22937,7 +22937,7 @@
       </c>
       <c r="H564" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -22962,7 +22962,7 @@
       </c>
       <c r="E565" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F565" s="7" t="inlineStr">
@@ -22977,7 +22977,7 @@
       </c>
       <c r="H565" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23002,7 +23002,7 @@
       </c>
       <c r="E566" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F566" s="7" t="inlineStr">
@@ -23017,7 +23017,7 @@
       </c>
       <c r="H566" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23042,7 +23042,7 @@
       </c>
       <c r="E567" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F567" s="7" t="inlineStr">
@@ -23057,7 +23057,7 @@
       </c>
       <c r="H567" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23082,7 +23082,7 @@
       </c>
       <c r="E568" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F568" s="7" t="inlineStr">
@@ -23097,7 +23097,7 @@
       </c>
       <c r="H568" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23122,7 +23122,7 @@
       </c>
       <c r="E569" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F569" s="7" t="inlineStr">
@@ -23137,7 +23137,7 @@
       </c>
       <c r="H569" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23162,7 +23162,7 @@
       </c>
       <c r="E570" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F570" s="7" t="inlineStr">
@@ -23177,7 +23177,7 @@
       </c>
       <c r="H570" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23202,7 +23202,7 @@
       </c>
       <c r="E571" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F571" s="7" t="inlineStr">
@@ -23217,7 +23217,7 @@
       </c>
       <c r="H571" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23242,7 +23242,7 @@
       </c>
       <c r="E572" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F572" s="7" t="inlineStr">
@@ -23257,7 +23257,7 @@
       </c>
       <c r="H572" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23282,7 +23282,7 @@
       </c>
       <c r="E573" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F573" s="7" t="inlineStr">
@@ -23297,7 +23297,7 @@
       </c>
       <c r="H573" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23322,7 +23322,7 @@
       </c>
       <c r="E574" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F574" s="7" t="inlineStr">
@@ -23337,7 +23337,7 @@
       </c>
       <c r="H574" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23362,7 +23362,7 @@
       </c>
       <c r="E575" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F575" s="7" t="inlineStr">
@@ -23377,7 +23377,7 @@
       </c>
       <c r="H575" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23402,7 +23402,7 @@
       </c>
       <c r="E576" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F576" s="7" t="inlineStr">
@@ -23417,7 +23417,7 @@
       </c>
       <c r="H576" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23442,7 +23442,7 @@
       </c>
       <c r="E577" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F577" s="7" t="inlineStr">
@@ -23457,7 +23457,7 @@
       </c>
       <c r="H577" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23482,7 +23482,7 @@
       </c>
       <c r="E578" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F578" s="7" t="inlineStr">
@@ -23497,7 +23497,7 @@
       </c>
       <c r="H578" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23522,7 +23522,7 @@
       </c>
       <c r="E579" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F579" s="7" t="inlineStr">
@@ -23537,7 +23537,7 @@
       </c>
       <c r="H579" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23562,7 +23562,7 @@
       </c>
       <c r="E580" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F580" s="7" t="inlineStr">
@@ -23577,7 +23577,7 @@
       </c>
       <c r="H580" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23602,7 +23602,7 @@
       </c>
       <c r="E581" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F581" s="7" t="inlineStr">
@@ -23617,7 +23617,7 @@
       </c>
       <c r="H581" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23642,7 +23642,7 @@
       </c>
       <c r="E582" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F582" s="7" t="inlineStr">
@@ -23657,7 +23657,7 @@
       </c>
       <c r="H582" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23682,7 +23682,7 @@
       </c>
       <c r="E583" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F583" s="7" t="inlineStr">
@@ -23697,7 +23697,7 @@
       </c>
       <c r="H583" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23722,7 +23722,7 @@
       </c>
       <c r="E584" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F584" s="7" t="inlineStr">
@@ -23737,7 +23737,7 @@
       </c>
       <c r="H584" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23762,7 +23762,7 @@
       </c>
       <c r="E585" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F585" s="7" t="inlineStr">
@@ -23777,7 +23777,7 @@
       </c>
       <c r="H585" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23802,7 +23802,7 @@
       </c>
       <c r="E586" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F586" s="7" t="inlineStr">
@@ -23817,7 +23817,7 @@
       </c>
       <c r="H586" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23842,7 +23842,7 @@
       </c>
       <c r="E587" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F587" s="7" t="inlineStr">
@@ -23857,7 +23857,7 @@
       </c>
       <c r="H587" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23882,7 +23882,7 @@
       </c>
       <c r="E588" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F588" s="7" t="inlineStr">
@@ -23897,7 +23897,7 @@
       </c>
       <c r="H588" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23922,7 +23922,7 @@
       </c>
       <c r="E589" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F589" s="7" t="inlineStr">
@@ -23937,7 +23937,7 @@
       </c>
       <c r="H589" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -23962,7 +23962,7 @@
       </c>
       <c r="E590" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F590" s="7" t="inlineStr">
@@ -23977,7 +23977,7 @@
       </c>
       <c r="H590" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24002,7 +24002,7 @@
       </c>
       <c r="E591" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F591" s="7" t="inlineStr">
@@ -24017,7 +24017,7 @@
       </c>
       <c r="H591" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24042,7 +24042,7 @@
       </c>
       <c r="E592" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F592" s="7" t="inlineStr">
@@ -24057,7 +24057,7 @@
       </c>
       <c r="H592" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24082,7 +24082,7 @@
       </c>
       <c r="E593" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F593" s="7" t="inlineStr">
@@ -24097,7 +24097,7 @@
       </c>
       <c r="H593" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24122,7 +24122,7 @@
       </c>
       <c r="E594" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F594" s="7" t="inlineStr">
@@ -24137,7 +24137,7 @@
       </c>
       <c r="H594" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24162,7 +24162,7 @@
       </c>
       <c r="E595" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F595" s="7" t="inlineStr">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="H595" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24202,7 +24202,7 @@
       </c>
       <c r="E596" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F596" s="7" t="inlineStr">
@@ -24217,7 +24217,7 @@
       </c>
       <c r="H596" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24242,7 +24242,7 @@
       </c>
       <c r="E597" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F597" s="7" t="inlineStr">
@@ -24257,7 +24257,7 @@
       </c>
       <c r="H597" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24282,7 +24282,7 @@
       </c>
       <c r="E598" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F598" s="7" t="inlineStr">
@@ -24297,7 +24297,7 @@
       </c>
       <c r="H598" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24322,7 +24322,7 @@
       </c>
       <c r="E599" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F599" s="7" t="inlineStr">
@@ -24337,7 +24337,7 @@
       </c>
       <c r="H599" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24362,7 +24362,7 @@
       </c>
       <c r="E600" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F600" s="7" t="inlineStr">
@@ -24377,7 +24377,7 @@
       </c>
       <c r="H600" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24402,7 +24402,7 @@
       </c>
       <c r="E601" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F601" s="7" t="inlineStr">
@@ -24417,7 +24417,7 @@
       </c>
       <c r="H601" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24442,7 +24442,7 @@
       </c>
       <c r="E602" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F602" s="7" t="inlineStr">
@@ -24457,7 +24457,7 @@
       </c>
       <c r="H602" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24482,7 +24482,7 @@
       </c>
       <c r="E603" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F603" s="7" t="inlineStr">
@@ -24497,7 +24497,7 @@
       </c>
       <c r="H603" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24522,7 +24522,7 @@
       </c>
       <c r="E604" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F604" s="7" t="inlineStr">
@@ -24537,7 +24537,7 @@
       </c>
       <c r="H604" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24562,7 +24562,7 @@
       </c>
       <c r="E605" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F605" s="7" t="inlineStr">
@@ -24577,7 +24577,7 @@
       </c>
       <c r="H605" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24602,7 +24602,7 @@
       </c>
       <c r="E606" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F606" s="7" t="inlineStr">
@@ -24617,7 +24617,7 @@
       </c>
       <c r="H606" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24642,7 +24642,7 @@
       </c>
       <c r="E607" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F607" s="7" t="inlineStr">
@@ -24657,7 +24657,7 @@
       </c>
       <c r="H607" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24682,7 +24682,7 @@
       </c>
       <c r="E608" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F608" s="7" t="inlineStr">
@@ -24697,7 +24697,7 @@
       </c>
       <c r="H608" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24722,7 +24722,7 @@
       </c>
       <c r="E609" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F609" s="7" t="inlineStr">
@@ -24737,7 +24737,7 @@
       </c>
       <c r="H609" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24762,7 +24762,7 @@
       </c>
       <c r="E610" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F610" s="7" t="inlineStr">
@@ -24777,7 +24777,7 @@
       </c>
       <c r="H610" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24802,7 +24802,7 @@
       </c>
       <c r="E611" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F611" s="7" t="inlineStr">
@@ -24817,7 +24817,7 @@
       </c>
       <c r="H611" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24842,7 +24842,7 @@
       </c>
       <c r="E612" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F612" s="7" t="inlineStr">
@@ -24857,7 +24857,7 @@
       </c>
       <c r="H612" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24882,7 +24882,7 @@
       </c>
       <c r="E613" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F613" s="7" t="inlineStr">
@@ -24897,7 +24897,7 @@
       </c>
       <c r="H613" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24922,7 +24922,7 @@
       </c>
       <c r="E614" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F614" s="7" t="inlineStr">
@@ -24937,7 +24937,7 @@
       </c>
       <c r="H614" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -24962,7 +24962,7 @@
       </c>
       <c r="E615" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F615" s="7" t="inlineStr">
@@ -24977,7 +24977,7 @@
       </c>
       <c r="H615" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25002,7 +25002,7 @@
       </c>
       <c r="E616" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F616" s="7" t="inlineStr">
@@ -25017,7 +25017,7 @@
       </c>
       <c r="H616" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25042,7 +25042,7 @@
       </c>
       <c r="E617" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F617" s="7" t="inlineStr">
@@ -25057,7 +25057,7 @@
       </c>
       <c r="H617" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25082,7 +25082,7 @@
       </c>
       <c r="E618" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F618" s="7" t="inlineStr">
@@ -25097,7 +25097,7 @@
       </c>
       <c r="H618" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25122,7 +25122,7 @@
       </c>
       <c r="E619" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F619" s="7" t="inlineStr">
@@ -25137,7 +25137,7 @@
       </c>
       <c r="H619" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25162,7 +25162,7 @@
       </c>
       <c r="E620" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F620" s="7" t="inlineStr">
@@ -25177,7 +25177,7 @@
       </c>
       <c r="H620" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25202,7 +25202,7 @@
       </c>
       <c r="E621" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F621" s="7" t="inlineStr">
@@ -25217,7 +25217,7 @@
       </c>
       <c r="H621" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25242,7 +25242,7 @@
       </c>
       <c r="E622" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F622" s="7" t="inlineStr">
@@ -25257,7 +25257,7 @@
       </c>
       <c r="H622" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25282,7 +25282,7 @@
       </c>
       <c r="E623" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F623" s="7" t="inlineStr">
@@ -25297,7 +25297,7 @@
       </c>
       <c r="H623" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25322,7 +25322,7 @@
       </c>
       <c r="E624" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F624" s="7" t="inlineStr">
@@ -25337,7 +25337,7 @@
       </c>
       <c r="H624" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25362,7 +25362,7 @@
       </c>
       <c r="E625" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F625" s="7" t="inlineStr">
@@ -25377,7 +25377,7 @@
       </c>
       <c r="H625" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25402,7 +25402,7 @@
       </c>
       <c r="E626" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F626" s="7" t="inlineStr">
@@ -25417,7 +25417,7 @@
       </c>
       <c r="H626" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25442,7 +25442,7 @@
       </c>
       <c r="E627" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F627" s="7" t="inlineStr">
@@ -25457,7 +25457,7 @@
       </c>
       <c r="H627" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25482,7 +25482,7 @@
       </c>
       <c r="E628" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F628" s="7" t="inlineStr">
@@ -25497,7 +25497,7 @@
       </c>
       <c r="H628" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25522,7 +25522,7 @@
       </c>
       <c r="E629" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F629" s="7" t="inlineStr">
@@ -25537,7 +25537,7 @@
       </c>
       <c r="H629" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25562,7 +25562,7 @@
       </c>
       <c r="E630" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F630" s="7" t="inlineStr">
@@ -25577,7 +25577,7 @@
       </c>
       <c r="H630" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25602,7 +25602,7 @@
       </c>
       <c r="E631" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F631" s="7" t="inlineStr">
@@ -25617,7 +25617,7 @@
       </c>
       <c r="H631" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25642,7 +25642,7 @@
       </c>
       <c r="E632" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F632" s="7" t="inlineStr">
@@ -25657,7 +25657,7 @@
       </c>
       <c r="H632" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25682,7 +25682,7 @@
       </c>
       <c r="E633" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F633" s="7" t="inlineStr">
@@ -25697,7 +25697,7 @@
       </c>
       <c r="H633" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25722,7 +25722,7 @@
       </c>
       <c r="E634" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F634" s="7" t="inlineStr">
@@ -25737,7 +25737,7 @@
       </c>
       <c r="H634" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25762,7 +25762,7 @@
       </c>
       <c r="E635" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F635" s="7" t="inlineStr">
@@ -25777,7 +25777,7 @@
       </c>
       <c r="H635" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25802,7 +25802,7 @@
       </c>
       <c r="E636" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F636" s="7" t="inlineStr">
@@ -25817,7 +25817,7 @@
       </c>
       <c r="H636" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25842,7 +25842,7 @@
       </c>
       <c r="E637" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F637" s="7" t="inlineStr">
@@ -25857,7 +25857,7 @@
       </c>
       <c r="H637" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25882,7 +25882,7 @@
       </c>
       <c r="E638" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F638" s="7" t="inlineStr">
@@ -25897,7 +25897,7 @@
       </c>
       <c r="H638" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25922,7 +25922,7 @@
       </c>
       <c r="E639" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F639" s="7" t="inlineStr">
@@ -25937,7 +25937,7 @@
       </c>
       <c r="H639" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -25962,7 +25962,7 @@
       </c>
       <c r="E640" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F640" s="7" t="inlineStr">
@@ -25977,7 +25977,7 @@
       </c>
       <c r="H640" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26002,7 +26002,7 @@
       </c>
       <c r="E641" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F641" s="7" t="inlineStr">
@@ -26017,7 +26017,7 @@
       </c>
       <c r="H641" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26042,7 +26042,7 @@
       </c>
       <c r="E642" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F642" s="7" t="inlineStr">
@@ -26057,7 +26057,7 @@
       </c>
       <c r="H642" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26082,7 +26082,7 @@
       </c>
       <c r="E643" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F643" s="7" t="inlineStr">
@@ -26097,7 +26097,7 @@
       </c>
       <c r="H643" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26122,7 +26122,7 @@
       </c>
       <c r="E644" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F644" s="7" t="inlineStr">
@@ -26137,7 +26137,7 @@
       </c>
       <c r="H644" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26162,7 +26162,7 @@
       </c>
       <c r="E645" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F645" s="7" t="inlineStr">
@@ -26177,7 +26177,7 @@
       </c>
       <c r="H645" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26202,7 +26202,7 @@
       </c>
       <c r="E646" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F646" s="7" t="inlineStr">
@@ -26217,7 +26217,7 @@
       </c>
       <c r="H646" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26242,7 +26242,7 @@
       </c>
       <c r="E647" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F647" s="7" t="inlineStr">
@@ -26257,7 +26257,7 @@
       </c>
       <c r="H647" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26282,7 +26282,7 @@
       </c>
       <c r="E648" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F648" s="7" t="inlineStr">
@@ -26297,7 +26297,7 @@
       </c>
       <c r="H648" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26322,7 +26322,7 @@
       </c>
       <c r="E649" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F649" s="7" t="inlineStr">
@@ -26337,7 +26337,7 @@
       </c>
       <c r="H649" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26362,7 +26362,7 @@
       </c>
       <c r="E650" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F650" s="7" t="inlineStr">
@@ -26377,7 +26377,7 @@
       </c>
       <c r="H650" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26402,7 +26402,7 @@
       </c>
       <c r="E651" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F651" s="7" t="inlineStr">
@@ -26417,7 +26417,7 @@
       </c>
       <c r="H651" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26442,7 +26442,7 @@
       </c>
       <c r="E652" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F652" s="7" t="inlineStr">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="H652" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26482,7 +26482,7 @@
       </c>
       <c r="E653" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F653" s="7" t="inlineStr">
@@ -26497,7 +26497,7 @@
       </c>
       <c r="H653" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26522,7 +26522,7 @@
       </c>
       <c r="E654" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F654" s="7" t="inlineStr">
@@ -26537,7 +26537,7 @@
       </c>
       <c r="H654" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26562,7 +26562,7 @@
       </c>
       <c r="E655" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F655" s="7" t="inlineStr">
@@ -26577,7 +26577,7 @@
       </c>
       <c r="H655" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26602,7 +26602,7 @@
       </c>
       <c r="E656" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F656" s="7" t="inlineStr">
@@ -26617,7 +26617,7 @@
       </c>
       <c r="H656" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26642,7 +26642,7 @@
       </c>
       <c r="E657" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F657" s="7" t="inlineStr">
@@ -26657,7 +26657,7 @@
       </c>
       <c r="H657" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26682,7 +26682,7 @@
       </c>
       <c r="E658" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F658" s="7" t="inlineStr">
@@ -26697,7 +26697,7 @@
       </c>
       <c r="H658" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26722,7 +26722,7 @@
       </c>
       <c r="E659" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F659" s="7" t="inlineStr">
@@ -26737,7 +26737,7 @@
       </c>
       <c r="H659" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26762,7 +26762,7 @@
       </c>
       <c r="E660" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F660" s="7" t="inlineStr">
@@ -26777,7 +26777,7 @@
       </c>
       <c r="H660" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26802,7 +26802,7 @@
       </c>
       <c r="E661" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F661" s="7" t="inlineStr">
@@ -26817,7 +26817,7 @@
       </c>
       <c r="H661" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26842,7 +26842,7 @@
       </c>
       <c r="E662" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F662" s="7" t="inlineStr">
@@ -26857,7 +26857,7 @@
       </c>
       <c r="H662" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26882,7 +26882,7 @@
       </c>
       <c r="E663" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F663" s="7" t="inlineStr">
@@ -26897,7 +26897,7 @@
       </c>
       <c r="H663" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26922,7 +26922,7 @@
       </c>
       <c r="E664" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F664" s="7" t="inlineStr">
@@ -26937,7 +26937,7 @@
       </c>
       <c r="H664" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -26962,7 +26962,7 @@
       </c>
       <c r="E665" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F665" s="7" t="inlineStr">
@@ -26977,7 +26977,7 @@
       </c>
       <c r="H665" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27002,7 +27002,7 @@
       </c>
       <c r="E666" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F666" s="7" t="inlineStr">
@@ -27017,7 +27017,7 @@
       </c>
       <c r="H666" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27042,7 +27042,7 @@
       </c>
       <c r="E667" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F667" s="7" t="inlineStr">
@@ -27057,7 +27057,7 @@
       </c>
       <c r="H667" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27082,7 +27082,7 @@
       </c>
       <c r="E668" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F668" s="7" t="inlineStr">
@@ -27097,7 +27097,7 @@
       </c>
       <c r="H668" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27122,7 +27122,7 @@
       </c>
       <c r="E669" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F669" s="7" t="inlineStr">
@@ -27137,7 +27137,7 @@
       </c>
       <c r="H669" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27162,7 +27162,7 @@
       </c>
       <c r="E670" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F670" s="7" t="inlineStr">
@@ -27177,7 +27177,7 @@
       </c>
       <c r="H670" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27202,7 +27202,7 @@
       </c>
       <c r="E671" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F671" s="7" t="inlineStr">
@@ -27217,7 +27217,7 @@
       </c>
       <c r="H671" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27242,7 +27242,7 @@
       </c>
       <c r="E672" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F672" s="7" t="inlineStr">
@@ -27257,7 +27257,7 @@
       </c>
       <c r="H672" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27282,7 +27282,7 @@
       </c>
       <c r="E673" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F673" s="7" t="inlineStr">
@@ -27297,7 +27297,7 @@
       </c>
       <c r="H673" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27322,7 +27322,7 @@
       </c>
       <c r="E674" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F674" s="7" t="inlineStr">
@@ -27337,7 +27337,7 @@
       </c>
       <c r="H674" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27362,7 +27362,7 @@
       </c>
       <c r="E675" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F675" s="7" t="inlineStr">
@@ -27377,7 +27377,7 @@
       </c>
       <c r="H675" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27402,7 +27402,7 @@
       </c>
       <c r="E676" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F676" s="7" t="inlineStr">
@@ -27417,7 +27417,7 @@
       </c>
       <c r="H676" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27442,7 +27442,7 @@
       </c>
       <c r="E677" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F677" s="7" t="inlineStr">
@@ -27457,7 +27457,7 @@
       </c>
       <c r="H677" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -27482,7 +27482,7 @@
       </c>
       <c r="E678" s="8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F678" s="7" t="inlineStr">
@@ -27497,7 +27497,7 @@
       </c>
       <c r="H678" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (PLANNER role): Skipped: submit disabled -- no product with an APPROVED price entry exists for this warehouse yet (needs Kế toán trưởng approval first, outside PLANNER's role) | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/price-history?status=APPROVED&amp;warehouseId=1 - Failed to load resource: the server responded with a status of 403 (Forbidden); http://localhost:3001/api/v1/price-history/lookup?productId=70&amp;warehouseId=1&amp;date=2026-07-25 - Failed to load resource: the server responded with a status of 404 (Not Found) (screenshot: OUT-004-round3.png)</t>
+          <t>Selenium E2E real business flow (PLANNER role): ok</t>
         </is>
       </c>
     </row>
@@ -32840,9 +32840,9 @@
           <t>Get All Periods Success</t>
         </is>
       </c>
-      <c r="E812" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E812" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F812" s="7" t="inlineStr">
@@ -32857,12 +32857,7 @@
       </c>
       <c r="H812" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -32885,9 +32880,9 @@
           <t>Create Period Success</t>
         </is>
       </c>
-      <c r="E813" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E813" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F813" s="7" t="inlineStr">
@@ -32902,12 +32897,7 @@
       </c>
       <c r="H813" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -32930,9 +32920,9 @@
           <t>Close Period Success</t>
         </is>
       </c>
-      <c r="E814" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E814" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F814" s="7" t="inlineStr">
@@ -32947,12 +32937,7 @@
       </c>
       <c r="H814" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -32975,9 +32960,9 @@
           <t>Get Active Notifications Success</t>
         </is>
       </c>
-      <c r="E815" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E815" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F815" s="7" t="inlineStr">
@@ -32992,12 +32977,7 @@
       </c>
       <c r="H815" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33020,9 +33000,9 @@
           <t>Mark As Read Success</t>
         </is>
       </c>
-      <c r="E816" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E816" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F816" s="7" t="inlineStr">
@@ -33037,12 +33017,7 @@
       </c>
       <c r="H816" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33065,9 +33040,9 @@
           <t>Create Invoice Accountant Returns201</t>
         </is>
       </c>
-      <c r="E817" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E817" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F817" s="7" t="inlineStr">
@@ -33082,12 +33057,7 @@
       </c>
       <c r="H817" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33110,9 +33080,9 @@
           <t>Create Invoice Storekeeper Returns403</t>
         </is>
       </c>
-      <c r="E818" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E818" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F818" s="7" t="inlineStr">
@@ -33127,12 +33097,7 @@
       </c>
       <c r="H818" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33155,9 +33120,9 @@
           <t>Get Invoices Accountant Returns200</t>
         </is>
       </c>
-      <c r="E819" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E819" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F819" s="7" t="inlineStr">
@@ -33172,12 +33137,7 @@
       </c>
       <c r="H819" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33200,9 +33160,9 @@
           <t>Create Payment Receipt Accountant Returns201</t>
         </is>
       </c>
-      <c r="E820" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E820" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F820" s="7" t="inlineStr">
@@ -33217,12 +33177,7 @@
       </c>
       <c r="H820" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33245,9 +33200,9 @@
           <t>Create Payment Receipt Storekeeper Returns403</t>
         </is>
       </c>
-      <c r="E821" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E821" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F821" s="7" t="inlineStr">
@@ -33262,12 +33217,7 @@
       </c>
       <c r="H821" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33290,9 +33240,9 @@
           <t>Get Payment Receipts Accountant Returns200</t>
         </is>
       </c>
-      <c r="E822" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E822" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F822" s="7" t="inlineStr">
@@ -33307,12 +33257,7 @@
       </c>
       <c r="H822" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33335,9 +33280,9 @@
           <t>Scan Payment Receipt Success</t>
         </is>
       </c>
-      <c r="E823" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E823" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F823" s="7" t="inlineStr">
@@ -33352,12 +33297,7 @@
       </c>
       <c r="H823" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33380,9 +33320,9 @@
           <t>Scan Payment Receipt Invalid File Type</t>
         </is>
       </c>
-      <c r="E824" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E824" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F824" s="7" t="inlineStr">
@@ -33397,12 +33337,7 @@
       </c>
       <c r="H824" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33425,9 +33360,9 @@
           <t>Create Supplier Invoice Success</t>
         </is>
       </c>
-      <c r="E825" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E825" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F825" s="7" t="inlineStr">
@@ -33442,12 +33377,7 @@
       </c>
       <c r="H825" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33470,9 +33400,9 @@
           <t>Get Supplier Invoices Success</t>
         </is>
       </c>
-      <c r="E826" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E826" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F826" s="7" t="inlineStr">
@@ -33487,12 +33417,7 @@
       </c>
       <c r="H826" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33515,9 +33440,9 @@
           <t>Get Supplier Invoice By Id Success</t>
         </is>
       </c>
-      <c r="E827" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E827" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F827" s="7" t="inlineStr">
@@ -33532,12 +33457,7 @@
       </c>
       <c r="H827" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33560,9 +33480,9 @@
           <t>Create Supplier Payment Success</t>
         </is>
       </c>
-      <c r="E828" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E828" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F828" s="7" t="inlineStr">
@@ -33577,12 +33497,7 @@
       </c>
       <c r="H828" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33605,9 +33520,9 @@
           <t>Get Supplier Payments Success</t>
         </is>
       </c>
-      <c r="E829" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E829" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F829" s="7" t="inlineStr">
@@ -33622,12 +33537,7 @@
       </c>
       <c r="H829" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33650,9 +33560,9 @@
           <t>Scan Supplier Payment Ocr Success</t>
         </is>
       </c>
-      <c r="E830" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E830" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F830" s="7" t="inlineStr">
@@ -33667,12 +33577,7 @@
       </c>
       <c r="H830" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33695,9 +33600,9 @@
           <t>Close Period Succeeds When No Pending Documents Exist</t>
         </is>
       </c>
-      <c r="E831" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E831" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F831" s="7" t="inlineStr">
@@ -33712,12 +33617,7 @@
       </c>
       <c r="H831" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33740,9 +33640,9 @@
           <t>Close Period Reports Blocking Receipts With Sample Numbers</t>
         </is>
       </c>
-      <c r="E832" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E832" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F832" s="7" t="inlineStr">
@@ -33757,12 +33657,7 @@
       </c>
       <c r="H832" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33785,9 +33680,9 @@
           <t>Close Period Rejects Already Closed Period</t>
         </is>
       </c>
-      <c r="E833" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E833" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F833" s="7" t="inlineStr">
@@ -33802,12 +33697,7 @@
       </c>
       <c r="H833" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33830,9 +33720,9 @@
           <t>Create Invoice Success</t>
         </is>
       </c>
-      <c r="E834" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E834" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F834" s="7" t="inlineStr">
@@ -33847,12 +33737,7 @@
       </c>
       <c r="H834" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33875,9 +33760,9 @@
           <t>Create Invoice Includes Pod Evidence From Delivery</t>
         </is>
       </c>
-      <c r="E835" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E835" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F835" s="7" t="inlineStr">
@@ -33892,12 +33777,7 @@
       </c>
       <c r="H835" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33920,9 +33800,9 @@
           <t>Create Invoice Denied For Non Accountant</t>
         </is>
       </c>
-      <c r="E836" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E836" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F836" s="7" t="inlineStr">
@@ -33937,12 +33817,7 @@
       </c>
       <c r="H836" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -33965,9 +33840,9 @@
           <t>Create Invoice Delivery Order Not Found</t>
         </is>
       </c>
-      <c r="E837" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E837" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F837" s="7" t="inlineStr">
@@ -33982,12 +33857,7 @@
       </c>
       <c r="H837" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34010,9 +33880,9 @@
           <t>Create Payment Receipt Success Fully Paid Unlocks Credit</t>
         </is>
       </c>
-      <c r="E838" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E838" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F838" s="7" t="inlineStr">
@@ -34027,12 +33897,7 @@
       </c>
       <c r="H838" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34055,9 +33920,9 @@
           <t>Run Daily Overdue Hold Job Locks Dealer And Alerts Accountant Managers</t>
         </is>
       </c>
-      <c r="E839" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E839" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F839" s="7" t="inlineStr">
@@ -34072,12 +33937,7 @@
       </c>
       <c r="H839" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34100,9 +33960,9 @@
           <t>Create Payment Receipt Denied For Non Accountant</t>
         </is>
       </c>
-      <c r="E840" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E840" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F840" s="7" t="inlineStr">
@@ -34117,12 +33977,7 @@
       </c>
       <c r="H840" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34145,9 +34000,9 @@
           <t>Create Payment Receipt Invoice Already Paid</t>
         </is>
       </c>
-      <c r="E841" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E841" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F841" s="7" t="inlineStr">
@@ -34162,12 +34017,7 @@
       </c>
       <c r="H841" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34190,9 +34040,9 @@
           <t>Create Payment Receipt Amount Exceeds Remaining</t>
         </is>
       </c>
-      <c r="E842" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E842" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F842" s="7" t="inlineStr">
@@ -34207,12 +34057,7 @@
       </c>
       <c r="H842" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34235,9 +34080,9 @@
           <t>Create Supplier Invoice Success</t>
         </is>
       </c>
-      <c r="E843" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E843" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F843" s="7" t="inlineStr">
@@ -34252,12 +34097,7 @@
       </c>
       <c r="H843" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34280,9 +34120,9 @@
           <t>Create Supplier Invoice Fails When Receipt Not Completed</t>
         </is>
       </c>
-      <c r="E844" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E844" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F844" s="7" t="inlineStr">
@@ -34297,12 +34137,7 @@
       </c>
       <c r="H844" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34325,9 +34160,9 @@
           <t>Create Supplier Invoice Fails For Non Accountant</t>
         </is>
       </c>
-      <c r="E845" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E845" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F845" s="7" t="inlineStr">
@@ -34342,12 +34177,7 @@
       </c>
       <c r="H845" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34370,9 +34200,9 @@
           <t>Create Supplier Payment Success</t>
         </is>
       </c>
-      <c r="E846" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E846" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F846" s="7" t="inlineStr">
@@ -34387,12 +34217,7 @@
       </c>
       <c r="H846" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34415,9 +34240,9 @@
           <t>Scan Supplier Payment Ocr Success</t>
         </is>
       </c>
-      <c r="E847" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E847" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F847" s="7" t="inlineStr">
@@ -34432,12 +34257,7 @@
       </c>
       <c r="H847" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34460,9 +34280,9 @@
           <t>Scan Supplier Payment Ocr Empty File Fails</t>
         </is>
       </c>
-      <c r="E848" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E848" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F848" s="7" t="inlineStr">
@@ -34477,12 +34297,7 @@
       </c>
       <c r="H848" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34505,9 +34320,9 @@
           <t>Create For Confirmed Delivery Creates Invoice Lines And Increases Dealer Balance</t>
         </is>
       </c>
-      <c r="E849" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E849" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F849" s="7" t="inlineStr">
@@ -34522,12 +34337,7 @@
       </c>
       <c r="H849" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34550,9 +34360,9 @@
           <t>Create For Confirmed Delivery Sets Due Date Thirty Days After Issue Date</t>
         </is>
       </c>
-      <c r="E850" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E850" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F850" s="7" t="inlineStr">
@@ -34567,12 +34377,7 @@
       </c>
       <c r="H850" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34595,9 +34400,9 @@
           <t>Create For Confirmed Delivery Rejects Missing Unit Price</t>
         </is>
       </c>
-      <c r="E851" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E851" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F851" s="7" t="inlineStr">
@@ -34612,12 +34417,7 @@
       </c>
       <c r="H851" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34640,9 +34440,9 @@
           <t>Create For Confirmed Delivery Returns Existing Invoice Without Balance Mutation</t>
         </is>
       </c>
-      <c r="E852" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E852" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F852" s="7" t="inlineStr">
@@ -34657,12 +34457,7 @@
       </c>
       <c r="H852" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34685,9 +34480,9 @@
           <t>Create For Confirmed Delivery Rejects Partial Delivery</t>
         </is>
       </c>
-      <c r="E853" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E853" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F853" s="7" t="inlineStr">
@@ -34702,12 +34497,7 @@
       </c>
       <c r="H853" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34730,9 +34520,9 @@
           <t>Create For Confirmed Delivery Handles Unique Constraint Collision Idempotently</t>
         </is>
       </c>
-      <c r="E854" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E854" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F854" s="7" t="inlineStr">
@@ -34747,12 +34537,7 @@
       </c>
       <c r="H854" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34775,9 +34560,9 @@
           <t>Create For Confirmed Delivery Audit Contains Dealer Balance Before And After</t>
         </is>
       </c>
-      <c r="E855" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E855" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F855" s="7" t="inlineStr">
@@ -34792,12 +34577,7 @@
       </c>
       <c r="H855" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34820,9 +34600,9 @@
           <t>Create For Confirmed Delivery Sets Credit Hold When Balance Exceeds Limit</t>
         </is>
       </c>
-      <c r="E856" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E856" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F856" s="7" t="inlineStr">
@@ -34837,12 +34617,7 @@
       </c>
       <c r="H856" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34865,9 +34640,9 @@
           <t>Create For Confirmed Delivery Stamps Accounting Period And Archives Billing Notification</t>
         </is>
       </c>
-      <c r="E857" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E857" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F857" s="7" t="inlineStr">
@@ -34882,12 +34657,7 @@
       </c>
       <c r="H857" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34910,9 +34680,9 @@
           <t>Create Backfill Invoice Rejects Delivery Order Not Completed</t>
         </is>
       </c>
-      <c r="E858" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E858" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F858" s="7" t="inlineStr">
@@ -34927,12 +34697,7 @@
       </c>
       <c r="H858" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -34955,9 +34720,9 @@
           <t>Create Backfill Invoice Rejects When Invoice Already Exists</t>
         </is>
       </c>
-      <c r="E859" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E859" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F859" s="7" t="inlineStr">
@@ -34972,12 +34737,7 @@
       </c>
       <c r="H859" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -35000,9 +34760,9 @@
           <t>Create Backfill Invoice Creates Invoice For Completed Order</t>
         </is>
       </c>
-      <c r="E860" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E860" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F860" s="7" t="inlineStr">
@@ -35017,12 +34777,7 @@
       </c>
       <c r="H860" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -35045,9 +34800,9 @@
           <t>renders accounting periods list correctly</t>
         </is>
       </c>
-      <c r="E861" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E861" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F861" s="7" t="inlineStr">
@@ -35062,12 +34817,7 @@
       </c>
       <c r="H861" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -35090,9 +34840,9 @@
           <t>opens confirmation modal and closes period on confirm</t>
         </is>
       </c>
-      <c r="E862" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E862" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F862" s="7" t="inlineStr">
@@ -35107,12 +34857,7 @@
       </c>
       <c r="H862" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -35135,9 +34880,9 @@
           <t>renders SupplierInvoices page and displays notification worklist</t>
         </is>
       </c>
-      <c r="E863" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E863" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F863" s="7" t="inlineStr">
@@ -35152,12 +34897,7 @@
       </c>
       <c r="H863" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -35180,9 +34920,9 @@
           <t>switches to Hóa đơn Mua hàng tab</t>
         </is>
       </c>
-      <c r="E864" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E864" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F864" s="7" t="inlineStr">
@@ -35197,12 +34937,7 @@
       </c>
       <c r="H864" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -35225,9 +34960,9 @@
           <t>opens modal to create supplier invoice when clicking Lập Hóa đơn Mua</t>
         </is>
       </c>
-      <c r="E865" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E865" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F865" s="7" t="inlineStr">
@@ -35242,12 +34977,7 @@
       </c>
       <c r="H865" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -35270,9 +35000,9 @@
           <t>renders title and invoices section</t>
         </is>
       </c>
-      <c r="E866" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E866" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F866" s="7" t="inlineStr">
@@ -35287,12 +35017,7 @@
       </c>
       <c r="H866" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -35315,9 +35040,9 @@
           <t>switches to aging report tab</t>
         </is>
       </c>
-      <c r="E867" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E867" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F867" s="7" t="inlineStr">
@@ -35332,12 +35057,7 @@
       </c>
       <c r="H867" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -35360,9 +35080,9 @@
           <t>renders title, form and payment log table</t>
         </is>
       </c>
-      <c r="E868" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E868" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F868" s="7" t="inlineStr">
@@ -35377,12 +35097,7 @@
       </c>
       <c r="H868" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -35405,9 +35120,9 @@
           <t>allows clicking record new payment button</t>
         </is>
       </c>
-      <c r="E869" s="9" t="inlineStr">
-        <is>
-          <t>Failed</t>
+      <c r="E869" s="8" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F869" s="7" t="inlineStr">
@@ -35422,12 +35137,7 @@
       </c>
       <c r="H869" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (ACCOUNTANT role): Error toast shown after submit: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/payment-receipts - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx 276:14 "Create AR payment failed:" AxiosError: OVERPAYMENT_EXCEEDS_INVOICE: OVERPAYMENT_EXCEEDS_INVOICE: Payment amount exceeds invoice remaining balance of 4000000.00
-    at settle (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1441:12)
-    at XMLHttpRequest.onloadend (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:1845:7)
-    at Axios.request (http://localhost:3001/node_modules/.vite/deps/axios.js?v=eeaa0ddc:2670:41)
-    at async Object.createPaymentReceipt (http://localhost:3001/src/services/finance.service.js:294:22)
-    at async handleSubmitPayment (http://localhost:3001/src/pages/Finance/DealerDebtInvoice.jsx:272:7) (screenshot: FIN-008-round3.png)</t>
+          <t>Selenium E2E real business flow (ACCOUNTANT role): ok</t>
         </is>
       </c>
     </row>
@@ -35467,7 +35177,7 @@
       </c>
       <c r="H870" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35507,7 +35217,7 @@
       </c>
       <c r="H871" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35547,7 +35257,7 @@
       </c>
       <c r="H872" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35587,7 +35297,7 @@
       </c>
       <c r="H873" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35627,7 +35337,7 @@
       </c>
       <c r="H874" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35667,7 +35377,7 @@
       </c>
       <c r="H875" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35707,7 +35417,7 @@
       </c>
       <c r="H876" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35747,7 +35457,7 @@
       </c>
       <c r="H877" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35787,7 +35497,7 @@
       </c>
       <c r="H878" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35827,7 +35537,7 @@
       </c>
       <c r="H879" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35867,7 +35577,7 @@
       </c>
       <c r="H880" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35907,7 +35617,7 @@
       </c>
       <c r="H881" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35947,7 +35657,7 @@
       </c>
       <c r="H882" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -35987,7 +35697,7 @@
       </c>
       <c r="H883" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36027,7 +35737,7 @@
       </c>
       <c r="H884" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36067,7 +35777,7 @@
       </c>
       <c r="H885" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36107,7 +35817,7 @@
       </c>
       <c r="H886" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36147,7 +35857,7 @@
       </c>
       <c r="H887" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36187,7 +35897,7 @@
       </c>
       <c r="H888" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36227,7 +35937,7 @@
       </c>
       <c r="H889" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36267,7 +35977,7 @@
       </c>
       <c r="H890" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36307,7 +36017,7 @@
       </c>
       <c r="H891" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36347,7 +36057,7 @@
       </c>
       <c r="H892" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36387,7 +36097,7 @@
       </c>
       <c r="H893" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36427,7 +36137,7 @@
       </c>
       <c r="H894" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36177,7 @@
       </c>
       <c r="H895" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36507,7 +36217,7 @@
       </c>
       <c r="H896" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36547,7 +36257,7 @@
       </c>
       <c r="H897" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36587,7 +36297,7 @@
       </c>
       <c r="H898" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36627,7 +36337,7 @@
       </c>
       <c r="H899" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36667,7 +36377,7 @@
       </c>
       <c r="H900" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36707,7 +36417,7 @@
       </c>
       <c r="H901" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36747,7 +36457,7 @@
       </c>
       <c r="H902" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36787,7 +36497,7 @@
       </c>
       <c r="H903" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36827,7 +36537,7 @@
       </c>
       <c r="H904" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36867,7 +36577,7 @@
       </c>
       <c r="H905" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36907,7 +36617,7 @@
       </c>
       <c r="H906" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36947,7 +36657,7 @@
       </c>
       <c r="H907" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -36987,7 +36697,7 @@
       </c>
       <c r="H908" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -37027,7 +36737,7 @@
       </c>
       <c r="H909" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -37067,7 +36777,7 @@
       </c>
       <c r="H910" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -37107,7 +36817,7 @@
       </c>
       <c r="H911" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -37147,7 +36857,7 @@
       </c>
       <c r="H912" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -37187,7 +36897,7 @@
       </c>
       <c r="H913" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -37227,7 +36937,7 @@
       </c>
       <c r="H914" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>
@@ -37267,7 +36977,7 @@
       </c>
       <c r="H915" s="7" t="inlineStr">
         <is>
-          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
+          <t>Selenium E2E real business flow (STOREKEEPER role): Error toast shown after submit: BUSINESS_RULE_VIOLATION: RETURN_EXCEEDS_ORIGINAL_SALE: Total returned quantity (2) exceeds original sales quantity (1.00) for product ID 11 | Console errors: http://localhost:3001/favicon.ico - Failed to load resource: the server responded with a status of 404 (Not Found); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity); http://localhost:3001/api/v1/returns - Failed to load resource: the server responded with a status of 422 (Unprocessable Entity) (screenshot: RET-009-round3.png)</t>
         </is>
       </c>
     </row>

</xml_diff>